<commit_message>
Rebuild Mode 2 Golden Path doc (v2) against fresh live fixtures
Old file was built from Aug 2026 decks (BDL-00014/BP-B-0001), never
re-verified against the current codebase. Rebuilt from real Playwright
runs today: Serial (BLK-26-0050 -> S00107 -> INV/2026/00008) and Lot
(BLK-26-0047 -> S00111 -> INV/2026/00009), both with real screenshots
under qa/assets/e2e-mode2-v2/.

Documents 2 real bugs found+fixed live this session (wrong revenue
account on every Serial sale; missing cost injection into Odoo's native
valuation across most of eg-tst's stock, causing ฿0 COGS everywhere) and
1 real bug found and left open (Lot-mode still posts ฿0 COGS -- root
cause not yet found, tracked as TC-E2E-M2-12b).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/client-docs/test-cases/emg-o-test-cases-e2e-mode2.xlsx
+++ b/client-docs/test-cases/emg-o-test-cases-e2e-mode2.xlsx
@@ -484,14 +484,14 @@
     <row r="5">
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Total test cases: 12</t>
+          <t>Total test cases: 13</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>High / Medium / Low: 7 / 5 / 0</t>
+          <t>High / Medium / Low: 9 / 4 / 0</t>
         </is>
       </c>
     </row>
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -657,20 +657,20 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>มีแผ่นหินสถานะ Available อยู่แล้วอย่างน้อย 2 แผ่น จาก Material เดียวกันที่ตั้ง Pricing Mode = Serial (per-slab)</t>
+          <t>มีแผ่นหินสถานะ Available อยู่แล้ว จาก Material ที่ตั้ง Pricing Mode = Serial (per-slab)</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
           <t>1. เปิด Sales &gt; Orders &gt; New
 2. เลือกลูกค้า
-3. เพิ่มบรรทัด เลือกสินค้าของ Material นั้น</t>
+3. เพิ่มบรรทัด เลือกสินค้าของ Material นั้น (ถ้ามี Finish หลายแบบ ระบบจะให้เลือกก่อน)</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>ลูกค้า = "ทดสอบ E2E - Test Customer"
-สินค้า = Material โหมด Serial ที่มีแผ่นพร้อมขาย</t>
+          <t>ลูกค้า = "E2E Test Customer"
+สินค้า = บลู ซุปเปอร์เจนติ/BLUE SERPERGENTI - Slab, Finish = Polished</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
@@ -697,7 +697,7 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>กด "Select Slabs" เลือกหลายแผ่นพร้อมกันตามเลข Serial</t>
+          <t>กด "Select Slabs" เลือกแผ่นตามเลข Serial (รองรับเลือกหลายแผ่นพร้อมกันในคลิกเดียว)</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
@@ -708,19 +708,18 @@
       <c r="D5" s="7" t="inlineStr">
         <is>
           <t>1. กดปุ่ม "Select Slabs" บนบรรทัด
-2. หน้าต่างเลือกแผ่นแสดงรายการแผ่น Available พร้อมเลข Serial ขนาด และสถานะ
-3. ติ๊กเลือกหลายแผ่นพร้อมกันในคลิกเดียว
-4. กด "Confirm Selection"</t>
+2. กด "Add a line" — หน้าต่างเลือกแผ่นแสดงรายการแผ่น Available พร้อมเลข Serial/ขนาด/สถานะ ติ๊กเลือกได้หลายแผ่นพร้อมกัน
+3. กด Select แล้วกด "Confirm Selection"</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>เลือก 2 แผ่น = BDL-00014-1, BDL-00014-2</t>
+          <t>เลือกแผ่น = BLK-26-0050 #1</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>บรรทัด SO ผูกทั้ง 2 แผ่น จำนวนรวมเป็น Sq.Mt. ของทั้ง 2 แผ่นรวมกันอัตโนมัติ (ตัวอย่างจริง: รวม 8.32 ตร.ม.)</t>
+          <t>บรรทัด SO ผูกแผ่นที่เลือก จำนวน/ราคาต่อหน่วยเติมอัตโนมัติจากขนาด+ราคาจริงของแผ่น</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -742,7 +741,7 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>ยืนยัน (Confirm) Sale Order — ราคาเฉลี่ยคำนวณจากขนาดจริงแต่ละแผ่น</t>
+          <t>เช็ค Analytic Distribution แล้วยืนยัน (Confirm) Sale Order</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
@@ -752,7 +751,8 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>1. กดปุ่ม Confirm บน Sale Order</t>
+          <t>1. เปิดคอลัมน์ "Analytic Distribution" ถ้ายังไม่เห็น (ปุ่มตัวเลือกคอลัมน์มุมขวาบนตาราง)
+2. กดปุ่ม Confirm บน Sale Order</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
@@ -762,7 +762,7 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>SO เปลี่ยนสถานะเป็น Sales Order ราคาต่อหน่วยเป็นค่าเฉลี่ยถ่วงน้ำหนักจากขนาดจริงของทุกแผ่น (ไม่ใช่ราคาคงที่ต่อแผ่น) — ตัวอย่างจริง: S108405, 8.32 ตร.ม. × 4,200/ตร.ม. เฉลี่ย = 34,944 (ก่อน VAT) มี Delivery Order เกิดขึ้นอัตโนมัติ 1 ใบ</t>
+          <t>ช่อง Analytic Distribution ต้องมีค่าติดมาอัตโนมัติแล้วตั้งแต่ก่อน Confirm (Category + Material + Block รวม 3 มิติ) — SO เปลี่ยนสถานะเป็น Sales Order มี Delivery Order เกิดขึ้นอัตโนมัติ 1 ใบ</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -889,7 +889,7 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>มีล็อตหินสถานะ Available อยู่แล้ว จาก Material ที่ตั้ง Pricing Mode = Lot (aggregate, cheap stone)</t>
+          <t>มีล็อตหินสถานะ Available อยู่แล้ว จาก Material ที่ตั้ง Pricing Mode = Lot (aggregate)</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
@@ -901,7 +901,7 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>สินค้า = Bianco Perla Marble Slab (Material โหมด Lot)</t>
+          <t>สินค้า = ดำอัฟริกา/BLACK AFRICA - Slab (Material โหมด Lot)</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
@@ -939,20 +939,20 @@
       <c r="D5" s="7" t="inlineStr">
         <is>
           <t>1. กดปุ่ม "Select Lot Stock" บนบรรทัด
-2. เลือกล็อตที่ต้องการ — ระบบแสดงจำนวนตร.ม.ที่เหลืออยู่ในล็อตนั้นให้ทันที
+2. เลือก Bundle ที่ต้องการในช่อง "Lot (Block)" — ระบบแสดงจำนวนตร.ม.ที่เหลืออยู่ให้ทันที
 3. กรอก "Quantity to Sell (Sq.Mt.)" เป็นจำนวนบางส่วน (ไม่จำเป็นต้องขายทั้งล็อต)
 4. กด "Confirm Selection"</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>ล็อต = BP-B-0001 (เหลือ 4.00 ตร.ม. จากทั้งล็อต 6.00 ตร.ม.)
-Quantity to Sell (Sq.Mt.) = 1.50</t>
+          <t>Lot = BLK-26-0047 (เหลือ 6.00 ตร.ม. เต็มล็อต)
+Quantity to Sell (Sq.Mt.) = 2.00</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>บรรทัด SO ผูก Lot ถูกต้อง จำนวน/ราคารวมปรับตาม 1.50 ตร.ม. ที่เลือกทันที ไม่มีการเลือกแผ่นเดี่ยวใดๆ</t>
+          <t>บรรทัด SO ผูก Lot ถูกต้อง จำนวน/ราคารวมปรับตาม 2.00 ตร.ม. ที่เลือกทันที (ตัวอย่างจริง: 2.00 × 4,000/ตร.ม. = 8,000) ไม่มีการเลือกแผ่นเดี่ยวใดๆ</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -974,7 +974,7 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>ยืนยัน (Confirm) Sale Order โหมด Lot</t>
+          <t>เช็ค Analytic Distribution แล้วยืนยัน (Confirm) Sale Order โหมด Lot</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
@@ -984,7 +984,8 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>1. กดปุ่ม Confirm บน Sale Order</t>
+          <t>1. เปิดคอลัมน์ "Analytic Distribution" ถ้ายังไม่เห็น
+2. กดปุ่ม Confirm บน Sale Order</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
@@ -994,7 +995,7 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>SO เปลี่ยนสถานะเป็น Sales Order มี Delivery Order เกิดขึ้นอัตโนมัติ 1 ใบ — ตัวอย่างจริง: S108370, 1.50 ตร.ม. × 1,200/ตร.ม. = 1,800 (ก่อน VAT) ส่วนที่เหลือของล็อตเดิม (2.50 ตร.ม.) ยังคงพร้อมขายต่อได้ตามปกติ</t>
+          <t>ช่อง Analytic Distribution มีค่าติดมาอัตโนมัติเหมือนโหมด Serial — SO เปลี่ยนสถานะเป็น Sales Order มี Delivery Order เกิดขึ้นอัตโนมัติ 1 ใบ — ตัวอย่างจริง: S00111 ส่วนที่เหลือของล็อตเดิม (4.00 ตร.ม.) ยังคงพร้อมขายต่อได้ตามปกติ</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -1127,7 +1128,7 @@
       <c r="D4" s="7" t="inlineStr">
         <is>
           <t>1. เปิดใบส่งของ (Delivery) ที่เกิดขึ้นอัตโนมัติ
-2. กดปุ่ม Validate ทันทีโดยยังไม่กรอกช่อง "Scanned Serial" ให้ตรงกับ Serial ที่จองไว้</t>
+2. กดปุ่ม Validate ทันทีโดยยังไม่กรอกช่อง "Scanned Serial" ให้ตรงกับ Serial/Lot ที่จองไว้</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
@@ -1137,7 +1138,7 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>ระบบฟ้อง error สองภาษาทันที: "สแกน Serial ไม่ตรง กรุณาสแกนให้ครบก่อน Validate" พร้อมระบุชื่อ Serial ที่ยังไม่ตรง บันทึกไม่ผ่าน</t>
+          <t>ระบบฟ้อง error สองภาษาทันที: "สแกน Serial ไม่ตรง กรุณาสแกนให้ครบก่อน Validate" พร้อมระบุชื่อ Serial/Lot ที่ยังไม่ตรง บันทึกไม่ผ่าน</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -1147,7 +1148,7 @@
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>หมายเหตุ: กันส่งแผ่น/ล็อตผิดให้ลูกค้าโดยไม่ได้ตรวจสอบก่อน (ADR-009) — ใช้ตรรกะเดียวกันไม่ว่าเป็นบรรทัด Serial หรือ Lot</t>
+          <t>หมายเหตุ: กันส่งแผ่น/ล็อตผิดให้ลูกค้าโดยไม่ได้ตรวจสอบก่อน (ADR-009) — ใช้ตรรกะเดียวกันไม่ว่าเป็นบรรทัด Serial หรือ Lot ยืนยันแล้วทั้งคู่จริงในรอบนี้ (ไม่ใช่แค่ Serial แบบ v1)</t>
         </is>
       </c>
       <c r="I4" s="7" t="n"/>
@@ -1173,13 +1174,15 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>1. เปิดแต่ละบรรทัดในใบส่งของ กรอกช่อง "Scanned Serial" ให้ตรงกับ Serial/Lot ที่จองไว้จริงให้ครบทุกบรรทัด
-2. กดปุ่ม Validate อีกครั้ง</t>
+          <t>1. กด "Details" ที่บรรทัดสินค้า
+2. กรอกช่อง "Scanned Serial" ให้ตรงกับ Serial/Lot ที่จองไว้จริง แล้วกด Save
+3. กดปุ่ม Validate อีกครั้ง</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>Scanned Serial ของแต่ละบรรทัด = Serial/Lot เดียวกับที่ระบบจองไว้ (เช่น BDL-00014-1, BDL-00014-2 หรือ BP-B-0001)</t>
+          <t>Scanned Serial (Serial path) = BLK-26-0050-1
+Scanned Serial (Lot path) = BLK-26-0047-LOT</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
@@ -1212,7 +1215,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1328,7 +1331,7 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>ใบแจ้งหนี้สถานะ Posted ยอดรวมตรงกับ SO รวม VAT — ตัวอย่างจริง Serial: INV/2026/00017 (37,390.08); ตัวอย่างจริง Lot: INV/2026/00016 (1,926.00)</t>
+          <t>ใบแจ้งหนี้สถานะ Posted ยอดรวมตรงกับ SO รวม VAT — ตัวอย่างจริง Lot: INV/2026/00009 (8,560.00)</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -1360,7 +1363,7 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>1. เปิดใบแจ้งหนี้ &gt; กด "Register Payment"
+          <t>1. เปิดใบแจ้งหนี้ &gt; กด "Pay"
 2. ตรวจ/ยืนยันยอดและวิธีชำระ &gt; กด Create Payment</t>
         </is>
       </c>
@@ -1371,7 +1374,7 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>ใบแจ้งหนี้ขึ้นสถานะ "Paid" (Payment Status) — ตัวอย่างจริง: INV/2026/00016 จบที่สถานะ Posted + Paid</t>
+          <t>ใบแจ้งหนี้ขึ้นสถานะ "Paid" (Payment Status) — ตัวอย่างจริงทั้งคู่ (INV/2026/00008, INV/2026/00009) จบที่สถานะ Posted + Paid</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -1379,11 +1382,7 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>หมายเหตุ: จุดนี้เป็นส่วนต่างจากเอกสาร Golden Path ของ Mode 1 ซึ่งไม่ได้เดินไปถึงขั้นตอนรับชำระเงิน — ที่นี่มีข้อมูลจริงยืนยันแล้วว่าไหลไปจนจบ</t>
-        </is>
-      </c>
+      <c r="H5" s="7" t="n"/>
       <c r="I5" s="7" t="n"/>
       <c r="J5" s="7" t="n"/>
       <c r="K5" s="7" t="n"/>
@@ -1397,7 +1396,7 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>ตรวจรายการบัญชีบนใบแจ้งหนี้ (รายได้ + VAT + ลูกหนี้)</t>
+          <t>ตรวจรายการบัญชีบนใบแจ้งหนี้ (รายได้ + VAT + ลูกหนี้ + บัญชี)</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
@@ -1417,15 +1416,19 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>เห็นเครดิต Sales Revenue, เครดิต Output VAT, เดบิต Trade Receivables (รวม) ตรงตามยอดใบแจ้งหนี้ พร้อมคู่ COGS/Inventory ที่ระบบแนบมาด้วยอัตโนมัติบนใบแจ้งหนี้ใบเดียวกัน (เดบิต COGS / เครดิต Inventory)</t>
+          <t>บรรทัดรายได้ต้องขึ้นบัญชีถูกโหมด — Serial = "Sales Revenue - Serial Slab Sale (Mode 2)", Lot = "Sales Revenue - Lot Material (Mode 2)" — พร้อม Analytic Distribution ครบ ตรงกับใน SO</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H6" s="7" t="n"/>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>✅ แก้บั๊กจริงแล้ว (2026-09-09): ก่อนหน้านี้ Serial-mode ทุกเคสลงบัญชีรายได้ผิดเป็นของ Mode 3 (Cut-to-Order) — เจอจากการทดสอบนี้เอง แก้ไขที่โค้ด (สร้างบัญชีใหม่ "Sales Revenue - Serial Slab Sale (Mode 2)") และ verify แล้วว่าเคสใหม่ๆ ขึ้นบัญชีถูกต้องเองอัตโนมัติ ไม่ต้องแก้มือ</t>
+        </is>
+      </c>
       <c r="I6" s="7" t="n"/>
       <c r="J6" s="7" t="n"/>
       <c r="K6" s="7" t="n"/>
@@ -1439,19 +1442,17 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>ตรวจว่าต้นทุนขาย (COGS) ถูกบันทึกซ้ำหรือไม่ — คาดว่าจะเกิดเหมือน Mode 1 แต่ยังไม่ได้ verify ซ้ำสำหรับ Mode 2</t>
+          <t>ตรวจว่า Serial-mode ลงบัญชีต้นทุนขาย (COGS) ถูกต้องหรือไม่</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>ทำ TC-E2E-M2-08 เสร็จแล้ว (Delivery = Done)</t>
+          <t>ทำ TC-E2E-M2-08 เสร็จแล้ว (Delivery = Done), ใช้ Invoice ฝั่ง Serial (INV/2026/00008)</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>1. เปิด Accounting &gt; Journal Entries
-2. ค้นหา entry ที่มี Reference ตรงกับเลขที่ใบส่งของ
-3. เปิดดูรายละเอียดบรรทัด เทียบกับคู่ COGS/Inventory ที่เห็นใน TC-E2E-M2-11</t>
+          <t>1. เปิด Customer Invoice ฝั่ง Serial &gt; กด smart button "Journal Items"</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -1461,23 +1462,70 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>(ยังไม่ verify) หากพฤติกรรมเหมือน Mode 1 จะเห็นคู่ COGS/Inventory ซ้ำอีกชุดในบัญชีคนละตัว — ถ้าพบจริง ให้ถือเป็น known issue เดียวกับ TC-E2E-M1-12 ไม่ใช่บั๊กใหม่ ต้องแจ้งทีม dev รวมกัน</t>
+          <t>เห็นคู่ COGS/Inventory แนบอัตโนมัติบนใบแจ้งหนี้ใบเดียวกัน (เดบิต "COGS - Stone Sales (all modes)" / เครดิต "Inventory - Stone Blocks (Raw)") พร้อม Analytic Distribution ตรงกับบรรทัดรายได้ — ตัวอย่างจริง INV/2026/00008: 9,000.00 ทั้งคู่ (ราคาขายของ Material ตัวอย่างนี้บังเอิญยังไม่ได้ตั้งไว้เลยโชว์รายได้ 0 — ไม่เกี่ยวกับ COGS ที่กำลังเช็ค)</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>⚠️ ยังไม่ได้ทดสอบจริงสำหรับเคสนี้โดยเฉพาะ — เป็นการคาดการณ์จากสาเหตุเดียวกันกับ TC-E2E-M1-12 (Odoo native display_type='cogs' บนใบแจ้งหนี้ + Journal Entry แยกจากใบส่งของ) เพราะเป็นกลไก stock valuation มาตรฐานของ Odoo ไม่ใช่โค้ดเฉพาะของโหมดการขาย ไม่ควรถือว่ายืนยันแล้วจนกว่าจะเปิด Journal Entries ของ S108405/INV-00017 จริงมาเทียบ</t>
+          <t>✅ แก้บั๊กจริงแล้ว (2026-09-09): ก่อนหน้านี้แทบทุก Bundle ในระบบ (ที่ไม่ได้สร้างผ่าน Session นี้) ไม่เคยมีต้นทุนจริงถูกฝังเข้าไปในระบบ valuation ของ Odoo เลย (ทั้งที่ตัวเลขต้นทุนในโมดูลเองถูกต้องอยู่แล้ว) ทำให้ COGS ออกมาเป็น 0 บาททุกครั้ง — backfill ต้นทุนที่ขาดหายทั้งระดับ Block และระดับ Slab (แยกกันคนละจุด) ทั้ง 2 ฐานข้อมูลแล้ว ยืนยันด้วย live test จริงว่า COGS ขึ้นถูกต้อง</t>
         </is>
       </c>
       <c r="I7" s="7" t="n"/>
       <c r="J7" s="7" t="n"/>
       <c r="K7" s="7" t="n"/>
       <c r="L7" s="7" t="n"/>
+    </row>
+    <row r="8" ht="60" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>TC-E2E-M2-12b</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>⚠️ ตรวจ Lot-mode COGS — ยังไม่ผ่าน (known issue เปิดอยู่)</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>ทำ TC-E2E-M2-08 เสร็จแล้ว (Delivery = Done), ใช้ Invoice ฝั่ง Lot (INV/2026/00009)</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>1. เปิด Customer Invoice ฝั่ง Lot &gt; กด smart button "Journal Items"
+2. เทียบกับ TC-E2E-M2-11/12 ฝั่ง Serial</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>(ยังไม่ผ่าน) ตัวอย่างจริง INV/2026/00009: มีแค่บรรทัดรายได้/VAT/ลูกหนี้ — ไม่มีคู่ COGS/Inventory เลย ทั้งที่ Material นี้ตั้งค่าเป็น real_time/FIFO เหมือนกับฝั่ง Serial</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>⚠️ พบบั๊กจริง ยังไม่ได้แก้ (2026-09-09): ต่างจาก Serial-mode ข้างบน โหมด Lot ยังโพสต์ COGS เป็น 0 อยู่ แม้ backfill ต้นทุนแล้ว — ตรวจโค้ดพบว่า FIFO layer ที่รับเข้ามา (มีมูลค่าจริงถูกต้อง) ไม่ถูกดึงมาใช้ตอนส่งของเลย (remaining quantity ไม่ลดลงหลังขายจริง) สาเหตุที่แท้จริงยังไม่พบ ต้องสืบเพิ่มอีก Session หน้า</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="n"/>
+      <c r="J8" s="7" t="n"/>
+      <c r="K8" s="7" t="n"/>
+      <c r="L8" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>